<commit_message>
removed test users from winners list
</commit_message>
<xml_diff>
--- a/outputs/final_consolation_winners_without_journals.xlsx
+++ b/outputs/final_consolation_winners_without_journals.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,144 +780,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Tihah Osman</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>853016431</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>25</v>
-      </c>
-      <c r="H5" t="n">
-        <v>25</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2026-04-11 20:22:45 GMT+8</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2026-02-19 11:27:07 GMT+8</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>no_journal_available</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>participant has no journal entries in Raw Journals</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Zaurida Ida</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>25770651572585175</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>25</v>
-      </c>
-      <c r="H6" t="n">
-        <v>25</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>2026-04-17 03:33:12 GMT+8</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2026-02-18 23:39:03 GMT+8</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>no_journal_available</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>participant has no journal entries in Raw Journals</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>